<commit_message>
Fix construction feed: fill missing 'Цена в валюте' field
Все 13 карточек ДСТ отклонены первой синхронизацией (отчёт
599059179): «Неправильно заполнен обязательный параметр — Цена
в валюте с НДС». Поле было в HEADERS, но не заполнялось в
build_row_excavator/build_row_bulldozer — тот же баг, что уже
чинился раньше в avito-feed/generate_feed.py (грузовики), не
перенёс исправление в новый скрипт. Теперь дублирует rec["price"]
в обеих функциях, как в остальных фидах.
</commit_message>
<xml_diff>
--- a/avito-feed-construction/fleet-construction.xlsx
+++ b/avito-feed-construction/fleet-construction.xlsx
@@ -842,7 +842,11 @@
         </is>
       </c>
       <c r="Z2" s="1" t="inlineStr"/>
-      <c r="AA2" s="1" t="inlineStr"/>
+      <c r="AA2" s="1" t="inlineStr">
+        <is>
+          <t>10800000</t>
+        </is>
+      </c>
       <c r="AB2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1002,7 +1006,11 @@
         </is>
       </c>
       <c r="Z3" s="1" t="inlineStr"/>
-      <c r="AA3" s="1" t="inlineStr"/>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>10800000</t>
+        </is>
+      </c>
       <c r="AB3" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1162,7 +1170,11 @@
         </is>
       </c>
       <c r="Z4" s="1" t="inlineStr"/>
-      <c r="AA4" s="1" t="inlineStr"/>
+      <c r="AA4" s="1" t="inlineStr">
+        <is>
+          <t>10800000</t>
+        </is>
+      </c>
       <c r="AB4" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1322,7 +1334,11 @@
         </is>
       </c>
       <c r="Z5" s="1" t="inlineStr"/>
-      <c r="AA5" s="1" t="inlineStr"/>
+      <c r="AA5" s="1" t="inlineStr">
+        <is>
+          <t>10800000</t>
+        </is>
+      </c>
       <c r="AB5" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1482,7 +1498,11 @@
         </is>
       </c>
       <c r="Z6" s="1" t="inlineStr"/>
-      <c r="AA6" s="1" t="inlineStr"/>
+      <c r="AA6" s="1" t="inlineStr">
+        <is>
+          <t>10000000</t>
+        </is>
+      </c>
       <c r="AB6" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1642,7 +1662,11 @@
         </is>
       </c>
       <c r="Z7" s="1" t="inlineStr"/>
-      <c r="AA7" s="1" t="inlineStr"/>
+      <c r="AA7" s="1" t="inlineStr">
+        <is>
+          <t>14500000</t>
+        </is>
+      </c>
       <c r="AB7" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1802,7 +1826,11 @@
         </is>
       </c>
       <c r="Z8" s="1" t="inlineStr"/>
-      <c r="AA8" s="1" t="inlineStr"/>
+      <c r="AA8" s="1" t="inlineStr">
+        <is>
+          <t>14500000</t>
+        </is>
+      </c>
       <c r="AB8" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1962,7 +1990,11 @@
         </is>
       </c>
       <c r="Z9" s="1" t="inlineStr"/>
-      <c r="AA9" s="1" t="inlineStr"/>
+      <c r="AA9" s="1" t="inlineStr">
+        <is>
+          <t>14500000</t>
+        </is>
+      </c>
       <c r="AB9" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -2122,7 +2154,11 @@
         </is>
       </c>
       <c r="Z10" s="1" t="inlineStr"/>
-      <c r="AA10" s="1" t="inlineStr"/>
+      <c r="AA10" s="1" t="inlineStr">
+        <is>
+          <t>14500000</t>
+        </is>
+      </c>
       <c r="AB10" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -2642,7 +2678,11 @@
         </is>
       </c>
       <c r="Z2" s="1" t="inlineStr"/>
-      <c r="AA2" s="1" t="inlineStr"/>
+      <c r="AA2" s="1" t="inlineStr">
+        <is>
+          <t>8800000</t>
+        </is>
+      </c>
       <c r="AB2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -2797,7 +2837,11 @@
         </is>
       </c>
       <c r="Z3" s="1" t="inlineStr"/>
-      <c r="AA3" s="1" t="inlineStr"/>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>8800000</t>
+        </is>
+      </c>
       <c r="AB3" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -2952,7 +2996,11 @@
         </is>
       </c>
       <c r="Z4" s="1" t="inlineStr"/>
-      <c r="AA4" s="1" t="inlineStr"/>
+      <c r="AA4" s="1" t="inlineStr">
+        <is>
+          <t>11800000</t>
+        </is>
+      </c>
       <c r="AB4" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -3443,7 +3491,11 @@
         </is>
       </c>
       <c r="Z2" s="1" t="inlineStr"/>
-      <c r="AA2" s="1" t="inlineStr"/>
+      <c r="AA2" s="1" t="inlineStr">
+        <is>
+          <t>19900000</t>
+        </is>
+      </c>
       <c r="AB2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>

</xml_diff>

<commit_message>
Fix construction feed: photo URLs missing /photos/ path segment
Все 13 карточек ДСТ в отчёте 599083414 получили 404 на все фото —
RAW_BASE в generate_feed.py указывал на .../avito-feed-construction/,
а файлы реально лежат в .../avito-feed-construction/photos/. Проверил
живьём (curl -I -> 200) перед пушем на этот раз.
</commit_message>
<xml_diff>
--- a/avito-feed-construction/fleet-construction.xlsx
+++ b/avito-feed-construction/fleet-construction.xlsx
@@ -815,7 +815,7 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>
@@ -979,7 +979,7 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -1307,7 +1307,7 @@
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="Q6" s="1" t="inlineStr"/>
       <c r="R6" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
         </is>
       </c>
       <c r="S6" s="1" t="inlineStr"/>
@@ -1635,7 +1635,7 @@
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
         </is>
       </c>
       <c r="S7" s="1" t="inlineStr"/>
@@ -1799,7 +1799,7 @@
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1963,7 +1963,7 @@
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
         </is>
       </c>
       <c r="S9" s="1" t="inlineStr"/>
@@ -2127,7 +2127,7 @@
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
         </is>
       </c>
       <c r="S10" s="1" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>
@@ -2810,7 +2810,7 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>
@@ -2969,7 +2969,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl621e/cff79444-c088-4e67-9215-e825d2b7c435.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jyl621e/376c62de-5217-4f96-9d27-8bd3fa1f4723.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl621e/cff79444-c088-4e67-9215-e825d2b7c435.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl621e/376c62de-5217-4f96-9d27-8bd3fa1f4723.JPG</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -3464,7 +3464,7 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy220c/43353c14-92c6-438c-a3d0-b4e19e3b9049.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy220c/ba477ea8-5aaf-496c-be56-55b5e465cf2b.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/jonyang-jy220c/8c27eb73-6266-41aa-9c02-f632a6236088.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy220c/43353c14-92c6-438c-a3d0-b4e19e3b9049.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy220c/ba477ea8-5aaf-496c-be56-55b5e465cf2b.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy220c/8c27eb73-6266-41aa-9c02-f632a6236088.JPG</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Remove nameplate/serial-number photos from construction feed
Артём попросил убрать все фото с VIN/серийным номером после
публикации. Убраны 3 фото шильдиков (JY625E, JY636E, JYL615F-E) —
у JYL621E и JY220C таких фото в фиде не было изначально. Проверил
все 52 оставшиеся ссылки на фото curl'ом перед пушем — все 200.
</commit_message>
<xml_diff>
--- a/avito-feed-construction/fleet-construction.xlsx
+++ b/avito-feed-construction/fleet-construction.xlsx
@@ -815,7 +815,7 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>
@@ -979,7 +979,7 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -1307,7 +1307,7 @@
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="Q6" s="1" t="inlineStr"/>
       <c r="R6" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/571d5749-f26e-41ee-9768-0cd7a2bdcff0.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/15891846-6c7e-418f-83d7-7fe2ca2cf4bb.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/5b8aed55-56e0-4cc2-aa27-32c4f33bddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy625e/f0fda440-4f99-4c22-b8e7-39c341d24c3d.JPG</t>
         </is>
       </c>
       <c r="S6" s="1" t="inlineStr"/>
@@ -1635,7 +1635,7 @@
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG</t>
         </is>
       </c>
       <c r="S7" s="1" t="inlineStr"/>
@@ -1799,7 +1799,7 @@
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1963,7 +1963,7 @@
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG</t>
         </is>
       </c>
       <c r="S9" s="1" t="inlineStr"/>
@@ -2127,7 +2127,7 @@
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/d5857bb6-b8f0-4fa4-ae50-1a110838b54f.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/4914ccf9-931d-4d22-9dac-be923fc1ddc8.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/eaaf0a0e-4b85-452e-b59c-f199cc8d0fe9.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/da0b4cb8-3556-4465-87e2-9c2ca93b79d2.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/89c5e118-02a9-4f8b-a9d9-448970a1c2c3.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/f5bc4d80-9e99-4e1e-b4f3-1fe18453c34c.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/26575e22-ad8a-4e04-b2d4-0e24d12569af.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jy636e/61050b30-ffbc-4861-a747-254a02538bba.JPG</t>
         </is>
       </c>
       <c r="S10" s="1" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>
@@ -2810,7 +2810,7 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/4ab5a6ca-48a0-4bdf-82e9-b37e2b4fc552.JPG</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/0d316b82-9b0e-4637-bafa-900ae468a21d.JPG | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-construction/photos/jonyang-jyl615fe/208fce80-93d8-4b35-b5f6-9d5ded06641e.JPG</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix phone number drifting back to default on every hourly sync
Feed always left "Номер телефона" empty, so Avito fell back to the
account default (79055945003) on each hourly re-sync, silently
undoing any manual phone change made in the Avito cabinet. Set an
explicit phone (79685590315, confirmed via listCompanyPhonesV1) on
all active records across all three feeds so it stays pinned.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/avito-feed-construction/fleet-construction.xlsx
+++ b/avito-feed-construction/fleet-construction.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гусеничные экскаваторы" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Колёсные экскаваторы" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бульдозеры" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Гусеничные экскаваторы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Колёсные экскаваторы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Бульдозеры" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -783,7 +783,11 @@
       <c r="E2" s="1" t="inlineStr"/>
       <c r="F2" s="1" t="inlineStr"/>
       <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -947,7 +951,11 @@
       <c r="E3" s="1" t="inlineStr"/>
       <c r="F3" s="1" t="inlineStr"/>
       <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1111,7 +1119,11 @@
       <c r="E4" s="1" t="inlineStr"/>
       <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr"/>
-      <c r="H4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1275,7 +1287,11 @@
       <c r="E5" s="1" t="inlineStr"/>
       <c r="F5" s="1" t="inlineStr"/>
       <c r="G5" s="1" t="inlineStr"/>
-      <c r="H5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1439,7 +1455,11 @@
       <c r="E6" s="1" t="inlineStr"/>
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1603,7 +1623,11 @@
       <c r="E7" s="1" t="inlineStr"/>
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1767,7 +1791,11 @@
       <c r="E8" s="1" t="inlineStr"/>
       <c r="F8" s="1" t="inlineStr"/>
       <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I8" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -1931,7 +1959,11 @@
       <c r="E9" s="1" t="inlineStr"/>
       <c r="F9" s="1" t="inlineStr"/>
       <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -2095,7 +2127,11 @@
       <c r="E10" s="1" t="inlineStr"/>
       <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr"/>
-      <c r="H10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -2619,7 +2655,11 @@
       <c r="E2" s="1" t="inlineStr"/>
       <c r="F2" s="1" t="inlineStr"/>
       <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -2778,7 +2818,11 @@
       <c r="E3" s="1" t="inlineStr"/>
       <c r="F3" s="1" t="inlineStr"/>
       <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -2937,7 +2981,11 @@
       <c r="E4" s="1" t="inlineStr"/>
       <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr"/>
-      <c r="H4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>
@@ -3432,7 +3480,11 @@
       <c r="E2" s="1" t="inlineStr"/>
       <c r="F2" s="1" t="inlineStr"/>
       <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>79685590315</t>
+        </is>
+      </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 15с2</t>

</xml_diff>